<commit_message>
feat: correção da main.py
</commit_message>
<xml_diff>
--- a/base_normalizada.xlsx
+++ b/base_normalizada.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DW84\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DW84\Downloads\manutencao_equipamentos-main-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{928CF376-4F68-4DEE-A7A7-D9836115DF52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{675C2D67-058F-4A60-A4EB-E155CB326A01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -353,8 +353,8 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabela1" displayName="Tabela1" ref="A1:L29">
   <autoFilter ref="A1:L29" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L20">
-    <sortCondition ref="G1:G20"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L29">
+    <sortCondition ref="G1:G29"/>
   </sortState>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Nº"/>
@@ -684,11 +684,11 @@
         <v>17</v>
       </c>
       <c r="J2">
-        <f t="shared" ref="J2:J14" si="0">ROUND((H2-G2)*24, 2)</f>
+        <f>ROUND((H2-G2)*24, 2)</f>
         <v>6</v>
       </c>
       <c r="K2" t="str">
-        <f t="shared" ref="K2:K25" si="1">IF(H2="","Aberto","Fechado")</f>
+        <f>IF(H2="","Aberto","Fechado")</f>
         <v>Fechado</v>
       </c>
       <c r="L2" s="3" t="str">
@@ -726,11 +726,11 @@
         <v>21</v>
       </c>
       <c r="J3">
-        <f t="shared" si="0"/>
+        <f>ROUND((H3-G3)*24, 2)</f>
         <v>25.33</v>
       </c>
       <c r="K3" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(H3="","Aberto","Fechado")</f>
         <v>Fechado</v>
       </c>
       <c r="L3" s="3" t="str">
@@ -768,15 +768,15 @@
         <v>22</v>
       </c>
       <c r="J4">
-        <f t="shared" si="0"/>
+        <f>ROUND((H4-G4)*24, 2)</f>
         <v>80.62</v>
       </c>
       <c r="K4" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(H4="","Aberto","Fechado")</f>
         <v>Fechado</v>
       </c>
       <c r="L4" s="3" t="str">
-        <f t="shared" ref="L4:L29" si="2">IF(OR(ISBLANK(G4),ISBLANK(H4)),"",IF(H4&lt;G4,"Data inválida",
+        <f>IF(OR(ISBLANK(G4),ISBLANK(H4)),"",IF(H4&lt;G4,"Data inválida",
 INT(H4-G4) &amp; " dias e " &amp; TEXT(H4-G4,"h") &amp; " horas"))</f>
         <v>3 dias e 8 horas</v>
       </c>
@@ -810,15 +810,16 @@
         <v>25</v>
       </c>
       <c r="J5">
-        <f t="shared" si="0"/>
+        <f>ROUND((H5-G5)*24, 2)</f>
         <v>0.87</v>
       </c>
       <c r="K5" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(H5="","Aberto","Fechado")</f>
         <v>Fechado</v>
       </c>
       <c r="L5" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(OR(ISBLANK(G5),ISBLANK(H5)),"",IF(H5&lt;G5,"Data inválida",
+INT(H5-G5) &amp; " dias e " &amp; TEXT(H5-G5,"h") &amp; " horas"))</f>
         <v>0 dias e 0 horas</v>
       </c>
     </row>
@@ -848,15 +849,16 @@
         <v>45811</v>
       </c>
       <c r="J6">
-        <f t="shared" si="0"/>
+        <f>ROUND((H6-G6)*24, 2)</f>
         <v>9.8000000000000007</v>
       </c>
       <c r="K6" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(H6="","Aberto","Fechado")</f>
         <v>Fechado</v>
       </c>
       <c r="L6" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(OR(ISBLANK(G6),ISBLANK(H6)),"",IF(H6&lt;G6,"Data inválida",
+INT(H6-G6) &amp; " dias e " &amp; TEXT(H6-G6,"h") &amp; " horas"))</f>
         <v>0 dias e 9 horas</v>
       </c>
     </row>
@@ -886,15 +888,16 @@
         <v>29</v>
       </c>
       <c r="J7">
-        <f t="shared" si="0"/>
+        <f>ROUND((H7-G7)*24, 2)</f>
         <v>312.72000000000003</v>
       </c>
       <c r="K7" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(H7="","Aberto","Fechado")</f>
         <v>Fechado</v>
       </c>
       <c r="L7" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(OR(ISBLANK(G7),ISBLANK(H7)),"",IF(H7&lt;G7,"Data inválida",
+INT(H7-G7) &amp; " dias e " &amp; TEXT(H7-G7,"h") &amp; " horas"))</f>
         <v>13 dias e 0 horas</v>
       </c>
     </row>
@@ -924,15 +927,16 @@
         <v>32</v>
       </c>
       <c r="J8">
-        <f t="shared" si="0"/>
+        <f>ROUND((H8-G8)*24, 2)</f>
         <v>5.75</v>
       </c>
       <c r="K8" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(H8="","Aberto","Fechado")</f>
         <v>Fechado</v>
       </c>
       <c r="L8" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(OR(ISBLANK(G8),ISBLANK(H8)),"",IF(H8&lt;G8,"Data inválida",
+INT(H8-G8) &amp; " dias e " &amp; TEXT(H8-G8,"h") &amp; " horas"))</f>
         <v>0 dias e 5 horas</v>
       </c>
     </row>
@@ -962,15 +966,16 @@
         <v>34</v>
       </c>
       <c r="J9">
-        <f t="shared" si="0"/>
+        <f>ROUND((H9-G9)*24, 2)</f>
         <v>30.9</v>
       </c>
       <c r="K9" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(H9="","Aberto","Fechado")</f>
         <v>Fechado</v>
       </c>
       <c r="L9" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(OR(ISBLANK(G9),ISBLANK(H9)),"",IF(H9&lt;G9,"Data inválida",
+INT(H9-G9) &amp; " dias e " &amp; TEXT(H9-G9,"h") &amp; " horas"))</f>
         <v>1 dias e 6 horas</v>
       </c>
     </row>
@@ -1000,15 +1005,16 @@
         <v>38</v>
       </c>
       <c r="J10">
-        <f t="shared" si="0"/>
+        <f>ROUND((H10-G10)*24, 2)</f>
         <v>120</v>
       </c>
       <c r="K10" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(H10="","Aberto","Fechado")</f>
         <v>Fechado</v>
       </c>
       <c r="L10" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(OR(ISBLANK(G10),ISBLANK(H10)),"",IF(H10&lt;G10,"Data inválida",
+INT(H10-G10) &amp; " dias e " &amp; TEXT(H10-G10,"h") &amp; " horas"))</f>
         <v>5 dias e 0 horas</v>
       </c>
     </row>
@@ -1038,15 +1044,16 @@
         <v>39</v>
       </c>
       <c r="J11">
-        <f t="shared" si="0"/>
+        <f>ROUND((H11-G11)*24, 2)</f>
         <v>31.5</v>
       </c>
       <c r="K11" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(H11="","Aberto","Fechado")</f>
         <v>Fechado</v>
       </c>
       <c r="L11" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(OR(ISBLANK(G11),ISBLANK(H11)),"",IF(H11&lt;G11,"Data inválida",
+INT(H11-G11) &amp; " dias e " &amp; TEXT(H11-G11,"h") &amp; " horas"))</f>
         <v>1 dias e 7 horas</v>
       </c>
     </row>
@@ -1076,15 +1083,16 @@
         <v>41</v>
       </c>
       <c r="J12">
-        <f t="shared" si="0"/>
+        <f>ROUND((H12-G12)*24, 2)</f>
         <v>30.5</v>
       </c>
       <c r="K12" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(H12="","Aberto","Fechado")</f>
         <v>Fechado</v>
       </c>
       <c r="L12" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(OR(ISBLANK(G12),ISBLANK(H12)),"",IF(H12&lt;G12,"Data inválida",
+INT(H12-G12) &amp; " dias e " &amp; TEXT(H12-G12,"h") &amp; " horas"))</f>
         <v>1 dias e 6 horas</v>
       </c>
     </row>
@@ -1114,15 +1122,16 @@
         <v>42</v>
       </c>
       <c r="J13">
-        <f t="shared" si="0"/>
+        <f>ROUND((H13-G13)*24, 2)</f>
         <v>88.5</v>
       </c>
       <c r="K13" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(H13="","Aberto","Fechado")</f>
         <v>Fechado</v>
       </c>
       <c r="L13" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(OR(ISBLANK(G13),ISBLANK(H13)),"",IF(H13&lt;G13,"Data inválida",
+INT(H13-G13) &amp; " dias e " &amp; TEXT(H13-G13,"h") &amp; " horas"))</f>
         <v>3 dias e 16 horas</v>
       </c>
     </row>
@@ -1152,15 +1161,16 @@
         <v>43</v>
       </c>
       <c r="J14">
-        <f t="shared" si="0"/>
+        <f>ROUND((H14-G14)*24, 2)</f>
         <v>57.65</v>
       </c>
       <c r="K14" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(H14="","Aberto","Fechado")</f>
         <v>Fechado</v>
       </c>
       <c r="L14" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(OR(ISBLANK(G14),ISBLANK(H14)),"",IF(H14&lt;G14,"Data inválida",
+INT(H14-G14) &amp; " dias e " &amp; TEXT(H14-G14,"h") &amp; " horas"))</f>
         <v>2 dias e 9 horas</v>
       </c>
     </row>
@@ -1188,11 +1198,12 @@
         <v>44</v>
       </c>
       <c r="K15" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(H15="","Aberto","Fechado")</f>
         <v>Aberto</v>
       </c>
       <c r="L15" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(OR(ISBLANK(G15),ISBLANK(H15)),"",IF(H15&lt;G15,"Data inválida",
+INT(H15-G15) &amp; " dias e " &amp; TEXT(H15-G15,"h") &amp; " horas"))</f>
         <v/>
       </c>
     </row>
@@ -1222,15 +1233,16 @@
         <v>45</v>
       </c>
       <c r="J16">
-        <f t="shared" ref="J16:J23" si="3">ROUND((H16-G16)*24, 2)</f>
+        <f>ROUND((H16-G16)*24, 2)</f>
         <v>339.3</v>
       </c>
       <c r="K16" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(H16="","Aberto","Fechado")</f>
         <v>Fechado</v>
       </c>
       <c r="L16" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(OR(ISBLANK(G16),ISBLANK(H16)),"",IF(H16&lt;G16,"Data inválida",
+INT(H16-G16) &amp; " dias e " &amp; TEXT(H16-G16,"h") &amp; " horas"))</f>
         <v>14 dias e 3 horas</v>
       </c>
     </row>
@@ -1260,15 +1272,16 @@
         <v>48</v>
       </c>
       <c r="J17">
-        <f t="shared" si="3"/>
+        <f>ROUND((H17-G17)*24, 2)</f>
         <v>41.5</v>
       </c>
       <c r="K17" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(H17="","Aberto","Fechado")</f>
         <v>Fechado</v>
       </c>
       <c r="L17" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(OR(ISBLANK(G17),ISBLANK(H17)),"",IF(H17&lt;G17,"Data inválida",
+INT(H17-G17) &amp; " dias e " &amp; TEXT(H17-G17,"h") &amp; " horas"))</f>
         <v>1 dias e 17 horas</v>
       </c>
     </row>
@@ -1298,97 +1311,100 @@
         <v>49</v>
       </c>
       <c r="J18">
-        <f t="shared" si="3"/>
+        <f>ROUND((H18-G18)*24, 2)</f>
         <v>82</v>
       </c>
       <c r="K18" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(H18="","Aberto","Fechado")</f>
         <v>Fechado</v>
       </c>
       <c r="L18" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(OR(ISBLANK(G18),ISBLANK(H18)),"",IF(H18&lt;G18,"Data inválida",
+INT(H18-G18) &amp; " dias e " &amp; TEXT(H18-G18,"h") &amp; " horas"))</f>
         <v>3 dias e 10 horas</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B19" t="s">
         <v>12</v>
       </c>
       <c r="C19" t="s">
-        <v>50</v>
+        <v>26</v>
       </c>
       <c r="E19" t="s">
-        <v>51</v>
+        <v>30</v>
       </c>
       <c r="F19" t="s">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="G19" s="2">
-        <v>45888.375</v>
+        <v>45884.708333333336</v>
       </c>
       <c r="H19" s="2">
-        <v>45910.625</v>
+        <v>45940.583333333336</v>
       </c>
       <c r="I19" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="J19">
-        <f t="shared" si="3"/>
-        <v>534</v>
+        <f>ROUND((H19-G19)*24, 2)</f>
+        <v>1341</v>
       </c>
       <c r="K19" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(H19="","Aberto","Fechado")</f>
         <v>Fechado</v>
       </c>
       <c r="L19" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>22 dias e 6 horas</v>
+        <f>IF(OR(ISBLANK(G19),ISBLANK(H19)),"",IF(H19&lt;G19,"Data inválida",
+INT(H19-G19) &amp; " dias e " &amp; TEXT(H19-G19,"h") &amp; " horas"))</f>
+        <v>55 dias e 21 horas</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B20" t="s">
         <v>12</v>
       </c>
       <c r="C20" t="s">
-        <v>26</v>
+        <v>50</v>
       </c>
       <c r="E20" t="s">
-        <v>30</v>
+        <v>51</v>
       </c>
       <c r="F20" t="s">
-        <v>33</v>
+        <v>52</v>
       </c>
       <c r="G20" s="2">
-        <v>45902.375</v>
+        <v>45888.375</v>
       </c>
       <c r="H20" s="2">
-        <v>45907.291666666664</v>
+        <v>45910.625</v>
       </c>
       <c r="I20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="J20">
-        <f t="shared" si="3"/>
-        <v>118</v>
+        <f>ROUND((H20-G20)*24, 2)</f>
+        <v>534</v>
       </c>
       <c r="K20" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(H20="","Aberto","Fechado")</f>
         <v>Fechado</v>
       </c>
       <c r="L20" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>4 dias e 22 horas</v>
+        <f>IF(OR(ISBLANK(G20),ISBLANK(H20)),"",IF(H20&lt;G20,"Data inválida",
+INT(H20-G20) &amp; " dias e " &amp; TEXT(H20-G20,"h") &amp; " horas"))</f>
+        <v>22 dias e 6 horas</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B21" t="s">
         <v>12</v>
@@ -1403,30 +1419,31 @@
         <v>33</v>
       </c>
       <c r="G21" s="2">
-        <v>45908.432638888888</v>
+        <v>45902.375</v>
       </c>
       <c r="H21" s="2">
-        <v>45916.4375</v>
+        <v>45907.291666666664</v>
       </c>
       <c r="I21" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="J21">
         <f>ROUND((H21-G21)*24, 2)</f>
-        <v>192.12</v>
+        <v>118</v>
       </c>
       <c r="K21" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(H21="","Aberto","Fechado")</f>
         <v>Fechado</v>
       </c>
       <c r="L21" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>8 dias e 0 horas</v>
+        <f>IF(OR(ISBLANK(G21),ISBLANK(H21)),"",IF(H21&lt;G21,"Data inválida",
+INT(H21-G21) &amp; " dias e " &amp; TEXT(H21-G21,"h") &amp; " horas"))</f>
+        <v>4 dias e 22 horas</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B22" t="s">
         <v>12</v>
@@ -1435,36 +1452,37 @@
         <v>26</v>
       </c>
       <c r="E22" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F22" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="G22" s="2">
-        <v>45924.333333333336</v>
+        <v>45908.432638888888</v>
       </c>
       <c r="H22" s="2">
-        <v>45945.333333333336</v>
-      </c>
-      <c r="I22" s="6" t="s">
-        <v>56</v>
+        <v>45916.4375</v>
+      </c>
+      <c r="I22" t="s">
+        <v>55</v>
       </c>
       <c r="J22">
-        <f t="shared" si="3"/>
-        <v>504</v>
+        <f>ROUND((H22-G22)*24, 2)</f>
+        <v>192.12</v>
       </c>
       <c r="K22" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(H22="","Aberto","Fechado")</f>
         <v>Fechado</v>
       </c>
       <c r="L22" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>21 dias e 0 horas</v>
+        <f>IF(OR(ISBLANK(G22),ISBLANK(H22)),"",IF(H22&lt;G22,"Data inválida",
+INT(H22-G22) &amp; " dias e " &amp; TEXT(H22-G22,"h") &amp; " horas"))</f>
+        <v>8 dias e 0 horas</v>
       </c>
     </row>
     <row r="23" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B23" t="s">
         <v>12</v>
@@ -1473,31 +1491,32 @@
         <v>26</v>
       </c>
       <c r="E23" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F23" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="G23" s="2">
-        <v>45884.708333333336</v>
+        <v>45924.333333333336</v>
       </c>
       <c r="H23" s="2">
-        <v>45940.583333333336</v>
-      </c>
-      <c r="I23" t="s">
-        <v>57</v>
+        <v>45945.333333333336</v>
+      </c>
+      <c r="I23" s="6" t="s">
+        <v>56</v>
       </c>
       <c r="J23">
-        <f t="shared" si="3"/>
-        <v>1341</v>
+        <f>ROUND((H23-G23)*24, 2)</f>
+        <v>504</v>
       </c>
       <c r="K23" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(H23="","Aberto","Fechado")</f>
         <v>Fechado</v>
       </c>
       <c r="L23" s="3" t="str">
-        <f t="shared" si="2"/>
-        <v>55 dias e 21 horas</v>
+        <f>IF(OR(ISBLANK(G23),ISBLANK(H23)),"",IF(H23&lt;G23,"Data inválida",
+INT(H23-G23) &amp; " dias e " &amp; TEXT(H23-G23,"h") &amp; " horas"))</f>
+        <v>21 dias e 0 horas</v>
       </c>
     </row>
     <row r="24" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1530,11 +1549,12 @@
         <v>96</v>
       </c>
       <c r="K24" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(H24="","Aberto","Fechado")</f>
         <v>Fechado</v>
       </c>
       <c r="L24" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(OR(ISBLANK(G24),ISBLANK(H24)),"",IF(H24&lt;G24,"Data inválida",
+INT(H24-G24) &amp; " dias e " &amp; TEXT(H24-G24,"h") &amp; " horas"))</f>
         <v>4 dias e 0 horas</v>
       </c>
     </row>
@@ -1568,11 +1588,12 @@
         <v>336.5</v>
       </c>
       <c r="K25" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(H25="","Aberto","Fechado")</f>
         <v>Fechado</v>
       </c>
       <c r="L25" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(OR(ISBLANK(G25),ISBLANK(H25)),"",IF(H25&lt;G25,"Data inválida",
+INT(H25-G25) &amp; " dias e " &amp; TEXT(H25-G25,"h") &amp; " horas"))</f>
         <v>14 dias e 0 horas</v>
       </c>
     </row>
@@ -1593,22 +1614,23 @@
         <v>40</v>
       </c>
       <c r="G26" s="2">
-        <v>45962.708333333336</v>
+        <v>45965.708333333336</v>
       </c>
       <c r="H26" s="2"/>
       <c r="I26" t="s">
         <v>61</v>
       </c>
       <c r="J26">
-        <f t="shared" ref="J26:J29" si="4">ROUND((H26-G26)*24, 2)</f>
-        <v>-1103105</v>
+        <f>ROUND((H26-G26)*24, 2)</f>
+        <v>-1103177</v>
       </c>
       <c r="K26" t="str">
         <f>IF(H26="","Aberto","Fechado")</f>
         <v>Aberto</v>
       </c>
       <c r="L26" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(OR(ISBLANK(G26),ISBLANK(H26)),"",IF(H26&lt;G26,"Data inválida",
+INT(H26-G26) &amp; " dias e " &amp; TEXT(H26-G26,"h") &amp; " horas"))</f>
         <v/>
       </c>
     </row>
@@ -1617,11 +1639,12 @@
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
       <c r="J27">
-        <f t="shared" si="4"/>
+        <f>ROUND((H27-G27)*24, 2)</f>
         <v>0</v>
       </c>
       <c r="L27" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(OR(ISBLANK(G27),ISBLANK(H27)),"",IF(H27&lt;G27,"Data inválida",
+INT(H27-G27) &amp; " dias e " &amp; TEXT(H27-G27,"h") &amp; " horas"))</f>
         <v/>
       </c>
     </row>
@@ -1629,11 +1652,12 @@
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
       <c r="J28">
-        <f t="shared" si="4"/>
+        <f>ROUND((H28-G28)*24, 2)</f>
         <v>0</v>
       </c>
       <c r="L28" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(OR(ISBLANK(G28),ISBLANK(H28)),"",IF(H28&lt;G28,"Data inválida",
+INT(H28-G28) &amp; " dias e " &amp; TEXT(H28-G28,"h") &amp; " horas"))</f>
         <v/>
       </c>
     </row>
@@ -1641,11 +1665,12 @@
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
       <c r="J29">
-        <f t="shared" si="4"/>
+        <f>ROUND((H29-G29)*24, 2)</f>
         <v>0</v>
       </c>
       <c r="L29" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f>IF(OR(ISBLANK(G29),ISBLANK(H29)),"",IF(H29&lt;G29,"Data inválida",
+INT(H29-G29) &amp; " dias e " &amp; TEXT(H29-G29,"h") &amp; " horas"))</f>
         <v/>
       </c>
     </row>
@@ -1662,12 +1687,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="078cfadf-81ba-4bd2-9020-6bf4b476ac98" xsi:nil="true"/>
+    <_Flow_SignoffStatus xmlns="cb4a64bd-25af-446c-a7d9-624a11665c21" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="cb4a64bd-25af-446c-a7d9-624a11665c21">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1918,21 +1946,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="078cfadf-81ba-4bd2-9020-6bf4b476ac98" xsi:nil="true"/>
-    <_Flow_SignoffStatus xmlns="cb4a64bd-25af-446c-a7d9-624a11665c21" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="cb4a64bd-25af-446c-a7d9-624a11665c21">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{050AFD69-4D1C-46C2-B506-AA5B8655C299}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{195248A8-5A8E-4D16-9204-5EE5D7659F2B}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="078cfadf-81ba-4bd2-9020-6bf4b476ac98"/>
+    <ds:schemaRef ds:uri="cb4a64bd-25af-446c-a7d9-624a11665c21"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1957,12 +1985,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{195248A8-5A8E-4D16-9204-5EE5D7659F2B}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{050AFD69-4D1C-46C2-B506-AA5B8655C299}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="078cfadf-81ba-4bd2-9020-6bf4b476ac98"/>
-    <ds:schemaRef ds:uri="cb4a64bd-25af-446c-a7d9-624a11665c21"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>